<commit_message>
Fold Whipping Cream into Class 1 milk, rename Ice Cream Mix to Ice Cream
Revenue & Profit Margin by Product: Whipping Cream no longer its own line,
now rolled into Class 1 milk (6 categories instead of 7); "Ice Cream Mix"
renamed to "Ice Cream" in both this chart and Cases by Product. Also fixes
the Revenue & Profit Margin by Product.xlsx template's "Overall Profit
Margin" formula, which was split across two cells by a stray comma and
never actually evaluated; it's now one formula with the corrected 6-row
range, wrapped in IFERROR so it reads 0 instead of #DIV/0! while blank.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/Revenue & Profit Margin by Product.xlsx
+++ b/data/Revenue & Profit Margin by Product.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -453,59 +453,47 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Whipping Cream</t>
+          <t>Ice Cream</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Ice Cream Mix</t>
+          <t>Soft Serve Mix</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Soft Serve Mix</t>
+          <t>Butter</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Butter</t>
+          <t>Sour Cream &amp; Chip Dip</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Sour Cream &amp; Chip Dip</t>
+          <t>Other (eggnog, co-packed)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Other (eggnog, co-packed)</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
           <t>Overall Profit Margin (weighted avg)</t>
         </is>
       </c>
-      <c r="C9">
-        <f>SUMPRODUCT(B2:B8</f>
+      <c r="C8">
+        <f>IFERROR(SUMPRODUCT(B2:B7,C2:C7)/SUM(B2:B7),0)</f>
         <v/>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>C2:C8)/SUM(B2:B8)</t>
-        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>